<commit_message>
feat: exported charts into outputs/
</commit_message>
<xml_diff>
--- a/01-equities-performance-analysis/outputs/summary_statistics.xlsx
+++ b/01-equities-performance-analysis/outputs/summary_statistics.xlsx
@@ -472,16 +472,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5021408227427804</v>
+        <v>0.005021408227427804</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1247836541016847</v>
+        <v>0.001247836541016847</v>
       </c>
       <c r="D2" t="n">
-        <v>2.10548142345924</v>
+        <v>0.0210548142345924</v>
       </c>
       <c r="E2" t="n">
-        <v>6.841386607077768</v>
+        <v>0.06841386607077768</v>
       </c>
       <c r="F2" t="n">
         <v>0.05926609121854378</v>
@@ -490,7 +490,7 @@
         <v>0.0002355055027742642</v>
       </c>
       <c r="H2" t="n">
-        <v>70.56074766355141</v>
+        <v>0.705607476635514</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.4364922616064915</v>
+        <v>0.004364922616064915</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1134777922579846</v>
+        <v>0.001134777922579846</v>
       </c>
       <c r="D3" t="n">
-        <v>2.203159068685914</v>
+        <v>0.02203159068685914</v>
       </c>
       <c r="E3" t="n">
-        <v>6.747107684795646</v>
+        <v>0.06747107684795646</v>
       </c>
       <c r="F3" t="n">
         <v>0.05150685389487971</v>
@@ -518,7 +518,7 @@
         <v>0.0004144094034182309</v>
       </c>
       <c r="H3" t="n">
-        <v>64.90696668109044</v>
+        <v>0.6490696668109044</v>
       </c>
     </row>
     <row r="4">
@@ -528,16 +528,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4810814608379843</v>
+        <v>0.004810814608379843</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1242528234671256</v>
+        <v>0.001242528234671256</v>
       </c>
       <c r="D4" t="n">
-        <v>2.27723293396939</v>
+        <v>0.0227723293396939</v>
       </c>
       <c r="E4" t="n">
-        <v>6.771243845251934</v>
+        <v>0.06771243845251934</v>
       </c>
       <c r="F4" t="n">
         <v>0.05456307153021168</v>
@@ -546,7 +546,7 @@
         <v>0.0004744306676422955</v>
       </c>
       <c r="H4" t="n">
-        <v>77.31818181818183</v>
+        <v>0.7731818181818183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>